<commit_message>
Fix stale Google Career jobs by inspecting page title in closure detection
</commit_message>
<xml_diff>
--- a/Job_Leads_Tracker.xlsx
+++ b/Job_Leads_Tracker.xlsx
@@ -74,7 +74,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +123,12 @@
         <bgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border/>
@@ -158,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -218,6 +224,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -495,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1025"/>
+  <dimension ref="A1:Z1038"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="19" customWidth="1" style="16" min="1" max="1"/>
@@ -5104,7 +5116,7 @@
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr">
@@ -5119,7 +5131,7 @@
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Automatically archived: job closed on careers portal.</t>
         </is>
       </c>
       <c r="K63" s="6" t="inlineStr">
@@ -5130,7 +5142,11 @@
       <c r="L63" s="3" t="n"/>
       <c r="M63" s="3" t="n"/>
       <c r="N63" s="3" t="n"/>
-      <c r="O63" s="3" t="n"/>
+      <c r="O63" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
       <c r="P63" s="3" t="n"/>
       <c r="Q63" s="3" t="n"/>
       <c r="R63" s="3" t="n"/>
@@ -5691,7 +5707,7 @@
           <t>Lead</t>
         </is>
       </c>
-      <c r="H71" s="8" t="inlineStr">
+      <c r="H71" s="23" t="inlineStr">
         <is>
           <t>Link to Job Description</t>
         </is>
@@ -5703,7 +5719,7 @@
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Direct link auto-updated/corrected via scan.</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
@@ -32958,7 +32974,7 @@
       </c>
       <c r="G1016" s="20" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="H1016" s="21" t="inlineStr">
@@ -32973,12 +32989,17 @@
       </c>
       <c r="J1016" s="19" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Automatically archived: job closed on careers portal.</t>
         </is>
       </c>
       <c r="K1016" s="19" t="inlineStr">
         <is>
           <t>$240,000 - $334,000</t>
+        </is>
+      </c>
+      <c r="O1016" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -33072,7 +33093,7 @@
       </c>
       <c r="G1018" s="20" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="H1018" s="21" t="inlineStr">
@@ -33087,12 +33108,17 @@
       </c>
       <c r="J1018" s="19" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Automatically archived: job closed on careers portal.</t>
         </is>
       </c>
       <c r="K1018" s="19" t="inlineStr">
         <is>
           <t>$240,000 - $334,000</t>
+        </is>
+      </c>
+      <c r="O1018" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -33129,7 +33155,7 @@
       </c>
       <c r="G1019" s="20" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="H1019" s="21" t="inlineStr">
@@ -33144,12 +33170,17 @@
       </c>
       <c r="J1019" s="19" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Automatically archived: job closed on careers portal.</t>
         </is>
       </c>
       <c r="K1019" s="19" t="inlineStr">
         <is>
           <t>$240,000 - $334,000</t>
+        </is>
+      </c>
+      <c r="O1019" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -33507,6 +33538,747 @@
       <c r="K1025" s="19" t="inlineStr">
         <is>
           <t>$192,000 - $240,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026" ht="22" customHeight="1" s="16">
+      <c r="A1026" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1026" s="22" t="inlineStr">
+        <is>
+          <t>Non-Mag 7</t>
+        </is>
+      </c>
+      <c r="C1026" s="19" t="inlineStr">
+        <is>
+          <t>Doordash</t>
+        </is>
+      </c>
+      <c r="D1026" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager, In-Store</t>
+        </is>
+      </c>
+      <c r="E1026" s="20" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="F1026" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1026" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1026" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1026" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1026" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1026" s="19" t="inlineStr">
+        <is>
+          <t>$159,800 - $235,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027" ht="22" customHeight="1" s="16">
+      <c r="A1027" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1027" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1027" s="19" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="D1027" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager, Ads Platform - Ads Reporting</t>
+        </is>
+      </c>
+      <c r="E1027" s="20" t="inlineStr">
+        <is>
+          <t>New York,New York,United States of America</t>
+        </is>
+      </c>
+      <c r="F1027" s="19" t="inlineStr">
+        <is>
+          <t>Netflix Phenom Portal crawl</t>
+        </is>
+      </c>
+      <c r="G1027" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1027" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1027" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1027" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1027" s="19" t="inlineStr">
+        <is>
+          <t>$310,000 - $545,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028" ht="22" customHeight="1" s="16">
+      <c r="A1028" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1028" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1028" s="19" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="D1028" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager, Ads Platform (Experimentation Foundations)</t>
+        </is>
+      </c>
+      <c r="E1028" s="20" t="inlineStr">
+        <is>
+          <t>Los Angeles,California,United States of America, Seattle,Washington,United States of America, New York,New York,United States of America, Los Gatos,California,United States of America</t>
+        </is>
+      </c>
+      <c r="F1028" s="19" t="inlineStr">
+        <is>
+          <t>Netflix Phenom Portal crawl</t>
+        </is>
+      </c>
+      <c r="G1028" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1028" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1028" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1028" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1028" s="19" t="inlineStr">
+        <is>
+          <t>$440,000 - $725,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029" ht="22" customHeight="1" s="16">
+      <c r="A1029" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1029" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1029" s="19" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1029" s="19" t="inlineStr">
+        <is>
+          <t>Principal Product Manager, Tech, Amazon Connect</t>
+        </is>
+      </c>
+      <c r="E1029" s="20" t="inlineStr">
+        <is>
+          <t>New York, New York, USA</t>
+        </is>
+      </c>
+      <c r="F1029" s="19" t="inlineStr">
+        <is>
+          <t>Amazon Public Search API (principal product manager)</t>
+        </is>
+      </c>
+      <c r="G1029" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1029" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1029" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1029" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1029" s="19" t="inlineStr">
+        <is>
+          <t>$199,200 - $269,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030" ht="22" customHeight="1" s="16">
+      <c r="A1030" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1030" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1030" s="19" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1030" s="19" t="inlineStr">
+        <is>
+          <t>Principal Product Manager - Tech, Creators and Social</t>
+        </is>
+      </c>
+      <c r="E1030" s="20" t="inlineStr">
+        <is>
+          <t>New York, New York, USA</t>
+        </is>
+      </c>
+      <c r="F1030" s="19" t="inlineStr">
+        <is>
+          <t>Amazon Public Search API (principal product manager)</t>
+        </is>
+      </c>
+      <c r="G1030" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1030" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1030" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1030" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1030" s="19" t="inlineStr">
+        <is>
+          <t>$197,900 - $267,800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031" ht="22" customHeight="1" s="16">
+      <c r="A1031" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1031" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1031" s="19" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1031" s="19" t="inlineStr">
+        <is>
+          <t>Principal Product Mgr. - Tech, Brand Measurement, Measurement, Ad Tech, and Data Science (MADS)</t>
+        </is>
+      </c>
+      <c r="E1031" s="20" t="inlineStr">
+        <is>
+          <t>New York, New York, USA</t>
+        </is>
+      </c>
+      <c r="F1031" s="19" t="inlineStr">
+        <is>
+          <t>Amazon Public Search API (principal product manager)</t>
+        </is>
+      </c>
+      <c r="G1031" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1031" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1031" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1031" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1031" s="19" t="inlineStr">
+        <is>
+          <t>$197,900 - $267,800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032" ht="22" customHeight="1" s="16">
+      <c r="A1032" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1032" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1032" s="19" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1032" s="19" t="inlineStr">
+        <is>
+          <t>Principal Product Mgr - Tech, Unified Auth, Unified Auth</t>
+        </is>
+      </c>
+      <c r="E1032" s="20" t="inlineStr">
+        <is>
+          <t>New York, New York, USA</t>
+        </is>
+      </c>
+      <c r="F1032" s="19" t="inlineStr">
+        <is>
+          <t>Amazon Public Search API (principal product manager)</t>
+        </is>
+      </c>
+      <c r="G1032" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1032" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1032" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1032" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1032" s="19" t="inlineStr">
+        <is>
+          <t>$197,900 - $267,800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033" ht="22" customHeight="1" s="16">
+      <c r="A1033" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1033" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs</t>
+        </is>
+      </c>
+      <c r="C1033" s="19" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="D1033" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager, Compute Platform</t>
+        </is>
+      </c>
+      <c r="E1033" s="20" t="inlineStr">
+        <is>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+        </is>
+      </c>
+      <c r="F1033" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1033" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1033" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1033" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1033" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1033" s="19" t="inlineStr">
+        <is>
+          <t>$305,000 - $385,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034" ht="22" customHeight="1" s="16">
+      <c r="A1034" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1034" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs</t>
+        </is>
+      </c>
+      <c r="C1034" s="19" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="D1034" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager, Enterprise</t>
+        </is>
+      </c>
+      <c r="E1034" s="20" t="inlineStr">
+        <is>
+          <t>San Francisco, CA | New York City, NY</t>
+        </is>
+      </c>
+      <c r="F1034" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1034" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1034" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1034" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1034" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1034" s="19" t="inlineStr">
+        <is>
+          <t>$385,000 - $595,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035" ht="22" customHeight="1" s="16">
+      <c r="A1035" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1035" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs</t>
+        </is>
+      </c>
+      <c r="C1035" s="19" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="D1035" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager, GTM Experiences</t>
+        </is>
+      </c>
+      <c r="E1035" s="20" t="inlineStr">
+        <is>
+          <t>San Francisco, CA | New York City, NY</t>
+        </is>
+      </c>
+      <c r="F1035" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1035" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1035" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1035" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1035" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1035" s="19" t="inlineStr">
+        <is>
+          <t>$305,000 - $385,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036" ht="22" customHeight="1" s="16">
+      <c r="A1036" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1036" s="22" t="inlineStr">
+        <is>
+          <t>Non-Mag 7</t>
+        </is>
+      </c>
+      <c r="C1036" s="19" t="inlineStr">
+        <is>
+          <t>Datadog</t>
+        </is>
+      </c>
+      <c r="D1036" s="19" t="inlineStr">
+        <is>
+          <t>Senior Product Manager, AAA/Enterprise Growth</t>
+        </is>
+      </c>
+      <c r="E1036" s="20" t="inlineStr">
+        <is>
+          <t>New York, New York, USA</t>
+        </is>
+      </c>
+      <c r="F1036" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1036" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1036" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1036" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1036" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1036" s="19" t="inlineStr">
+        <is>
+          <t>$192,000 - $240,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037" ht="22" customHeight="1" s="16">
+      <c r="A1037" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1037" s="22" t="inlineStr">
+        <is>
+          <t>Non-Mag 7</t>
+        </is>
+      </c>
+      <c r="C1037" s="19" t="inlineStr">
+        <is>
+          <t>Datadog</t>
+        </is>
+      </c>
+      <c r="D1037" s="19" t="inlineStr">
+        <is>
+          <t>Senior Product Manager, SQL &amp; Sheets Growth</t>
+        </is>
+      </c>
+      <c r="E1037" s="20" t="inlineStr">
+        <is>
+          <t>New York, New York, USA</t>
+        </is>
+      </c>
+      <c r="F1037" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1037" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1037" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1037" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1037" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1037" s="19" t="inlineStr">
+        <is>
+          <t>$187,000 - $240,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038" ht="22" customHeight="1" s="16">
+      <c r="A1038" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1038" s="22" t="inlineStr">
+        <is>
+          <t>Non-Mag 7</t>
+        </is>
+      </c>
+      <c r="C1038" s="19" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D1038" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager Project Intern (Brand Advertising - Monetization Product) - 2026 Start (BS/MS)</t>
+        </is>
+      </c>
+      <c r="E1038" s="20" t="inlineStr">
+        <is>
+          <t>New York, New York</t>
+        </is>
+      </c>
+      <c r="F1038" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via TikTok automated API sync</t>
+        </is>
+      </c>
+      <c r="G1038" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1038" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1038" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="J1038" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1038" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -33616,6 +34388,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1023" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1024" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1025" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1026" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1027" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1028" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1029" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1030" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1031" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1032" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1033" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1034" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1035" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1036" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1037" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1038" r:id="rId117"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
Consolidate 'AI Labs' and 'High-Growth Startups' cohorts and integrate 16 new technology startup scrapers
</commit_message>
<xml_diff>
--- a/Job_Leads_Tracker.xlsx
+++ b/Job_Leads_Tracker.xlsx
@@ -164,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -230,6 +230,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -507,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1038"/>
+  <dimension ref="A1:Z1059"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="19" customWidth="1" style="16" min="1" max="1"/>
@@ -617,9 +620,9 @@
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>AI Labs</t>
+      <c r="B2" s="25" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -1873,9 +1876,9 @@
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>High-Growth Startups</t>
+      <c r="B19" s="25" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -1945,9 +1948,9 @@
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>High-Growth Startups</t>
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -2021,9 +2024,9 @@
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>High-Growth Startups</t>
+      <c r="B21" s="25" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -2093,9 +2096,9 @@
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>High-Growth Startups</t>
+      <c r="B22" s="25" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -2165,9 +2168,9 @@
           <t>[x]</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>AI Labs</t>
+      <c r="B23" s="25" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -2947,7 +2950,7 @@
           <t>Lead</t>
         </is>
       </c>
-      <c r="H33" s="8" t="inlineStr">
+      <c r="H33" s="23" t="inlineStr">
         <is>
           <t>Link to Job Description</t>
         </is>
@@ -2959,7 +2962,7 @@
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Direct link auto-updated/corrected via scan.</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -3637,9 +3640,9 @@
           <t>[ ]</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>AI Labs</t>
+      <c r="B43" s="25" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -4464,7 +4467,7 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr">
@@ -4479,7 +4482,7 @@
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Automatically archived: job closed on careers portal.</t>
         </is>
       </c>
       <c r="K54" s="6" t="inlineStr">
@@ -4490,7 +4493,11 @@
       <c r="L54" s="3" t="n"/>
       <c r="M54" s="3" t="n"/>
       <c r="N54" s="3" t="n"/>
-      <c r="O54" s="3" t="n"/>
+      <c r="O54" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
       <c r="P54" s="3" t="n"/>
       <c r="Q54" s="3" t="n"/>
       <c r="R54" s="3" t="n"/>
@@ -4536,7 +4543,7 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="H55" s="8" t="inlineStr">
@@ -4551,7 +4558,7 @@
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Automatically archived: job closed on careers portal.</t>
         </is>
       </c>
       <c r="K55" s="6" t="inlineStr">
@@ -4562,7 +4569,11 @@
       <c r="L55" s="3" t="n"/>
       <c r="M55" s="3" t="n"/>
       <c r="N55" s="3" t="n"/>
-      <c r="O55" s="3" t="n"/>
+      <c r="O55" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
       <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n"/>
       <c r="R55" s="3" t="n"/>
@@ -4972,7 +4983,7 @@
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr">
@@ -4987,7 +4998,7 @@
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Automatically archived: job closed on careers portal.</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr">
@@ -4998,7 +5009,11 @@
       <c r="L61" s="3" t="n"/>
       <c r="M61" s="3" t="n"/>
       <c r="N61" s="3" t="n"/>
-      <c r="O61" s="3" t="n"/>
+      <c r="O61" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
       <c r="P61" s="3" t="n"/>
       <c r="Q61" s="3" t="n"/>
       <c r="R61" s="3" t="n"/>
@@ -5264,7 +5279,7 @@
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="H65" s="8" t="inlineStr">
@@ -5279,7 +5294,7 @@
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Automatically archived: job closed on careers portal.</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr">
@@ -5290,7 +5305,11 @@
       <c r="L65" s="3" t="n"/>
       <c r="M65" s="3" t="n"/>
       <c r="N65" s="3" t="n"/>
-      <c r="O65" s="3" t="n"/>
+      <c r="O65" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
       <c r="P65" s="3" t="n"/>
       <c r="Q65" s="3" t="n"/>
       <c r="R65" s="3" t="n"/>
@@ -31943,7 +31962,7 @@
       </c>
       <c r="G998" s="20" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="H998" s="21" t="inlineStr">
@@ -31958,12 +31977,17 @@
       </c>
       <c r="J998" s="19" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Automatically archived: job closed on careers portal.</t>
         </is>
       </c>
       <c r="K998" s="19" t="inlineStr">
         <is>
           <t>$166,300 - $225,000</t>
+        </is>
+      </c>
+      <c r="O998" s="0" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -32057,7 +32081,7 @@
       </c>
       <c r="G1000" s="20" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="H1000" s="21" t="inlineStr">
@@ -32072,12 +32096,17 @@
       </c>
       <c r="J1000" s="19" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Automatically archived: job closed on careers portal.</t>
         </is>
       </c>
       <c r="K1000" s="19" t="inlineStr">
         <is>
           <t>$152,200 - $206,000</t>
+        </is>
+      </c>
+      <c r="O1000" s="0" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -32305,7 +32334,7 @@
       </c>
       <c r="J1004" s="19" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Direct link auto-updated/corrected via scan.</t>
         </is>
       </c>
       <c r="K1004" s="19" t="inlineStr">
@@ -32997,7 +33026,7 @@
           <t>$240,000 - $334,000</t>
         </is>
       </c>
-      <c r="O1016" t="inlineStr">
+      <c r="O1016" s="0" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -33116,7 +33145,7 @@
           <t>$240,000 - $334,000</t>
         </is>
       </c>
-      <c r="O1018" t="inlineStr">
+      <c r="O1018" s="0" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -33178,7 +33207,7 @@
           <t>$240,000 - $334,000</t>
         </is>
       </c>
-      <c r="O1019" t="inlineStr">
+      <c r="O1019" s="0" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -33217,7 +33246,7 @@
       </c>
       <c r="G1020" s="20" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="H1020" s="21" t="inlineStr">
@@ -33232,12 +33261,17 @@
       </c>
       <c r="J1020" s="19" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Automatically archived: job closed on careers portal.</t>
         </is>
       </c>
       <c r="K1020" s="19" t="inlineStr">
         <is>
           <t>$256,000 - $278,000</t>
+        </is>
+      </c>
+      <c r="O1020" s="0" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -33948,7 +33982,7 @@
       </c>
       <c r="B1033" s="24" t="inlineStr">
         <is>
-          <t>AI Labs</t>
+          <t>AI Labs &amp; Startups</t>
         </is>
       </c>
       <c r="C1033" s="19" t="inlineStr">
@@ -34005,7 +34039,7 @@
       </c>
       <c r="B1034" s="24" t="inlineStr">
         <is>
-          <t>AI Labs</t>
+          <t>AI Labs &amp; Startups</t>
         </is>
       </c>
       <c r="C1034" s="19" t="inlineStr">
@@ -34030,7 +34064,7 @@
       </c>
       <c r="G1034" s="20" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="H1034" s="21" t="inlineStr">
@@ -34045,12 +34079,17 @@
       </c>
       <c r="J1034" s="19" t="inlineStr">
         <is>
-          <t>Discovered by daily scan.</t>
+          <t>Automatically archived: job closed on careers portal.</t>
         </is>
       </c>
       <c r="K1034" s="19" t="inlineStr">
         <is>
           <t>$385,000 - $595,000</t>
+        </is>
+      </c>
+      <c r="O1034" s="0" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -34062,7 +34101,7 @@
       </c>
       <c r="B1035" s="24" t="inlineStr">
         <is>
-          <t>AI Labs</t>
+          <t>AI Labs &amp; Startups</t>
         </is>
       </c>
       <c r="C1035" s="19" t="inlineStr">
@@ -34273,12 +34312,1209 @@
       </c>
       <c r="J1038" s="19" t="inlineStr">
         <is>
+          <t>Direct link auto-updated/corrected via scan.</t>
+        </is>
+      </c>
+      <c r="K1038" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039" ht="22" customHeight="1" s="16">
+      <c r="A1039" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1039" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1039" s="19" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="D1039" s="19" t="inlineStr">
+        <is>
+          <t>Senior Product Manager, Generative AI, Google Cloud</t>
+        </is>
+      </c>
+      <c r="E1039" s="20" t="inlineStr">
+        <is>
+          <t>Kirkland, WA, USA, New York, NY, USA, Sunnyvale, CA, USA, San Francisco, CA, USA</t>
+        </is>
+      </c>
+      <c r="F1039" s="19" t="inlineStr">
+        <is>
+          <t>Google Careers HTML crawl (Senior product manager)</t>
+        </is>
+      </c>
+      <c r="G1039" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1039" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1039" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1039" s="19" t="inlineStr">
+        <is>
           <t>Discovered by daily scan.</t>
         </is>
       </c>
-      <c r="K1038" s="19" t="inlineStr">
+      <c r="K1039" s="19" t="inlineStr">
+        <is>
+          <t>$192,000 - $279,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040" ht="22" customHeight="1" s="16">
+      <c r="A1040" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1040" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1040" s="19" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="D1040" s="19" t="inlineStr">
+        <is>
+          <t>Group Product Manager, YouTube Live Events</t>
+        </is>
+      </c>
+      <c r="E1040" s="20" t="inlineStr">
+        <is>
+          <t>San Bruno, CA, USA, Cambridge, MA, USA, New York, NY, USA, Los Angeles, CA, USA</t>
+        </is>
+      </c>
+      <c r="F1040" s="19" t="inlineStr">
+        <is>
+          <t>Google Careers HTML crawl (Senior product manager)</t>
+        </is>
+      </c>
+      <c r="G1040" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1040" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1040" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1040" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1040" s="19" t="inlineStr">
+        <is>
+          <t>$240,000 - $334,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041" ht="22" customHeight="1" s="16">
+      <c r="A1041" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1041" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1041" s="19" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="D1041" s="19" t="inlineStr">
+        <is>
+          <t>Group Product Manager, Generative Media, Google Labs</t>
+        </is>
+      </c>
+      <c r="E1041" s="20" t="inlineStr">
+        <is>
+          <t>Mountain View, CA, USA, New York, NY, USA</t>
+        </is>
+      </c>
+      <c r="F1041" s="19" t="inlineStr">
+        <is>
+          <t>Google Careers HTML crawl (Senior product manager)</t>
+        </is>
+      </c>
+      <c r="G1041" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1041" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1041" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1041" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1041" s="19" t="inlineStr">
+        <is>
+          <t>$240,000 - $334,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042" ht="22" customHeight="1" s="16">
+      <c r="A1042" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1042" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1042" s="19" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1042" s="19" t="inlineStr">
+        <is>
+          <t>Principal Product Manager - Technical, Ads AI Core Infrastructure</t>
+        </is>
+      </c>
+      <c r="E1042" s="20" t="inlineStr">
+        <is>
+          <t>New York, New York, USA</t>
+        </is>
+      </c>
+      <c r="F1042" s="19" t="inlineStr">
+        <is>
+          <t>Amazon Public Search API (principal product manager)</t>
+        </is>
+      </c>
+      <c r="G1042" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1042" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1042" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1042" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1042" s="19" t="inlineStr">
+        <is>
+          <t>$197,900 - $267,800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043" ht="22" customHeight="1" s="16">
+      <c r="A1043" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1043" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1043" s="19" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1043" s="19" t="inlineStr">
+        <is>
+          <t>Principal. Product Manager - Tech, Measurement Ad Tech Data Science</t>
+        </is>
+      </c>
+      <c r="E1043" s="20" t="inlineStr">
+        <is>
+          <t>New York, New York, USA</t>
+        </is>
+      </c>
+      <c r="F1043" s="19" t="inlineStr">
+        <is>
+          <t>Amazon Public Search API (principal product manager)</t>
+        </is>
+      </c>
+      <c r="G1043" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1043" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1043" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1043" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1043" s="19" t="inlineStr">
+        <is>
+          <t>$197,900 - $267,800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044" ht="22" customHeight="1" s="16">
+      <c r="A1044" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1044" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1044" s="19" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D1044" s="19" t="inlineStr">
+        <is>
+          <t>Principal PMT, Sponsored Products</t>
+        </is>
+      </c>
+      <c r="E1044" s="20" t="inlineStr">
+        <is>
+          <t>New York, New York, USA</t>
+        </is>
+      </c>
+      <c r="F1044" s="19" t="inlineStr">
+        <is>
+          <t>Amazon Public Search API (principal product manager)</t>
+        </is>
+      </c>
+      <c r="G1044" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1044" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1044" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1044" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1044" s="19" t="inlineStr">
+        <is>
+          <t>$197,900 - $267,800</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045" ht="22" customHeight="1" s="16">
+      <c r="A1045" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1045" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1045" s="19" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="D1045" s="19" t="inlineStr">
+        <is>
+          <t>Product Management, Human Data Platform</t>
+        </is>
+      </c>
+      <c r="E1045" s="20" t="inlineStr">
+        <is>
+          <t>San Francisco, CA | New York City, NY</t>
+        </is>
+      </c>
+      <c r="F1045" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1045" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1045" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1045" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1045" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1045" s="19" t="inlineStr">
+        <is>
+          <t>$305,000 - $385,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046" ht="22" customHeight="1" s="16">
+      <c r="A1046" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1046" s="18" t="inlineStr">
+        <is>
+          <t>Mag 7</t>
+        </is>
+      </c>
+      <c r="C1046" s="19" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D1046" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager - Experimentation Platform</t>
+        </is>
+      </c>
+      <c r="E1046" s="20" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="F1046" s="19" t="inlineStr">
+        <is>
+          <t>Apple Careers HTML crawl</t>
+        </is>
+      </c>
+      <c r="G1046" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1046" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1046" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1046" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1046" s="19" t="inlineStr">
+        <is>
+          <t>$181,100 - $272,100</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047" ht="22" customHeight="1" s="16">
+      <c r="A1047" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1047" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1047" s="19" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="D1047" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager | Agentic CX</t>
+        </is>
+      </c>
+      <c r="E1047" s="20" t="inlineStr">
+        <is>
+          <t>New York, NY (HQ)</t>
+        </is>
+      </c>
+      <c r="F1047" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Ashby automated crawl</t>
+        </is>
+      </c>
+      <c r="G1047" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1047" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1047" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1047" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1047" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048" ht="22" customHeight="1" s="16">
+      <c r="A1048" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1048" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1048" s="19" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="D1048" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager | Generalist (All Levels)</t>
+        </is>
+      </c>
+      <c r="E1048" s="20" t="inlineStr">
+        <is>
+          <t>New York, NY (HQ)</t>
+        </is>
+      </c>
+      <c r="F1048" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Ashby automated crawl</t>
+        </is>
+      </c>
+      <c r="G1048" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1048" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1048" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1048" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1048" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049" ht="22" customHeight="1" s="16">
+      <c r="A1049" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1049" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1049" s="19" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="D1049" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager | Vendor Intelligence &amp; Marketplace</t>
+        </is>
+      </c>
+      <c r="E1049" s="20" t="inlineStr">
+        <is>
+          <t>New York, NY (HQ)</t>
+        </is>
+      </c>
+      <c r="F1049" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Ashby automated crawl</t>
+        </is>
+      </c>
+      <c r="G1049" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1049" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1049" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1049" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1049" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050" ht="22" customHeight="1" s="16">
+      <c r="A1050" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1050" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1050" s="19" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="D1050" s="19" t="inlineStr">
+        <is>
+          <t>Director of Product Management, Forward Deployed &amp; Strategy</t>
+        </is>
+      </c>
+      <c r="E1050" s="20" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="F1050" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1050" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1050" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1050" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1050" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1050" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051" ht="22" customHeight="1" s="16">
+      <c r="A1051" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1051" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1051" s="19" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="D1051" s="19" t="inlineStr">
+        <is>
+          <t>Forward Deployed Product Manager, Enterprise</t>
+        </is>
+      </c>
+      <c r="E1051" s="20" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="F1051" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1051" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1051" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1051" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1051" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1051" s="19" t="inlineStr">
+        <is>
+          <t>$205,600 - $300,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052" ht="22" customHeight="1" s="16">
+      <c r="A1052" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1052" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1052" s="19" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="D1052" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager, Data Engine</t>
+        </is>
+      </c>
+      <c r="E1052" s="20" t="inlineStr">
+        <is>
+          <t>San Francisco, CA; St. Louis, MO; New York, NY; Washington, DC</t>
+        </is>
+      </c>
+      <c r="F1052" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1052" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1052" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1052" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1052" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1052" s="19" t="inlineStr">
+        <is>
+          <t>$205,600 - $257,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053" ht="22" customHeight="1" s="16">
+      <c r="A1053" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1053" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1053" s="19" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="D1053" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager, Enterprise Core Platform</t>
+        </is>
+      </c>
+      <c r="E1053" s="20" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="F1053" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1053" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1053" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1053" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1053" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1053" s="19" t="inlineStr">
+        <is>
+          <t>$205,600 - $300,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054" ht="22" customHeight="1" s="16">
+      <c r="A1054" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1054" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1054" s="19" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="D1054" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager, Gen AI</t>
+        </is>
+      </c>
+      <c r="E1054" s="20" t="inlineStr">
+        <is>
+          <t>New York, NY; San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="F1054" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1054" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1054" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1054" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1054" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1054" s="19" t="inlineStr">
+        <is>
+          <t>$205,600 - $257,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055" ht="22" customHeight="1" s="16">
+      <c r="A1055" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1055" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1055" s="19" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="D1055" s="19" t="inlineStr">
+        <is>
+          <t>Product Manager, Public Sector GenAI Test &amp; Evaluation (T&amp;E)</t>
+        </is>
+      </c>
+      <c r="E1055" s="20" t="inlineStr">
+        <is>
+          <t>San Francisco, CA; St. Louis, MO; New York, NY; Washington, DC</t>
+        </is>
+      </c>
+      <c r="F1055" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1055" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1055" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1055" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1055" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1055" s="19" t="inlineStr">
+        <is>
+          <t>$205,600 - $257,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056" ht="22" customHeight="1" s="16">
+      <c r="A1056" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1056" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1056" s="19" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="D1056" s="19" t="inlineStr">
+        <is>
+          <t>Staff Product Manager, Agentic Platform</t>
+        </is>
+      </c>
+      <c r="E1056" s="20" t="inlineStr">
+        <is>
+          <t>New York, NY; San Francisco, CA; Washington, DC</t>
+        </is>
+      </c>
+      <c r="F1056" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1056" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1056" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1056" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1056" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1056" s="19" t="inlineStr">
+        <is>
+          <t>$237,600 - $297,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057" ht="22" customHeight="1" s="16">
+      <c r="A1057" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1057" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1057" s="19" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="D1057" s="19" t="inlineStr">
+        <is>
+          <t>Staff Technical Product Manager</t>
+        </is>
+      </c>
+      <c r="E1057" s="20" t="inlineStr">
+        <is>
+          <t>London, UK; New York, NY; San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="F1057" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Greenhouse automated crawl</t>
+        </is>
+      </c>
+      <c r="G1057" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1057" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1057" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1057" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1057" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058" ht="22" customHeight="1" s="16">
+      <c r="A1058" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1058" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1058" s="19" t="inlineStr">
+        <is>
+          <t>Harvey</t>
+        </is>
+      </c>
+      <c r="D1058" s="19" t="inlineStr">
+        <is>
+          <t>Staff Product Manager, New Verticals</t>
+        </is>
+      </c>
+      <c r="E1058" s="20" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F1058" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Ashby automated crawl</t>
+        </is>
+      </c>
+      <c r="G1058" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1058" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1058" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1058" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1058" s="19" t="inlineStr">
+        <is>
+          <t>$215,000 - $300,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059" ht="22" customHeight="1" s="16">
+      <c r="A1059" s="17" t="inlineStr">
+        <is>
+          <t>[ ]</t>
+        </is>
+      </c>
+      <c r="B1059" s="24" t="inlineStr">
+        <is>
+          <t>AI Labs &amp; Startups</t>
+        </is>
+      </c>
+      <c r="C1059" s="19" t="inlineStr">
+        <is>
+          <t>Harvey</t>
+        </is>
+      </c>
+      <c r="D1059" s="19" t="inlineStr">
+        <is>
+          <t>Innovation Product Manager</t>
+        </is>
+      </c>
+      <c r="E1059" s="20" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F1059" s="19" t="inlineStr">
+        <is>
+          <t>Discovered via Ashby automated crawl</t>
+        </is>
+      </c>
+      <c r="G1059" s="20" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="H1059" s="21" t="inlineStr">
+        <is>
+          <t>Link to Job Description</t>
+        </is>
+      </c>
+      <c r="I1059" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="J1059" s="19" t="inlineStr">
+        <is>
+          <t>Discovered by daily scan.</t>
+        </is>
+      </c>
+      <c r="K1059" s="19" t="inlineStr">
+        <is>
+          <t>$178,500 - $241,500</t>
         </is>
       </c>
     </row>
@@ -34401,6 +35637,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1036" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1037" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1038" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1039" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1040" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1041" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1042" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1043" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1044" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1045" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1046" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1047" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1048" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1049" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1050" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1051" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1052" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1053" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1054" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1055" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1056" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1057" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1058" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1059" r:id="rId138"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>